<commit_message>
ajustes de titulos, textos e conclusões
</commit_message>
<xml_diff>
--- a/dataset/raw/base_relatorios_llm.xlsx
+++ b/dataset/raw/base_relatorios_llm.xlsx
@@ -480,11 +480,11 @@
         </is>
       </c>
       <c r="G2" t="n">
-        <v>62.82</v>
+        <v>62.39</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Erro ao gerar relatório clínico: Failed to connect to Ollama. Please check that Ollama is downloaded, running and accessible. https://ollama.com/download</t>
+          <t>Com base nos dados fornecidos – glicose de 140 mg/dL, IMC de 32 e idade de 45 anos – o modelo de diagnóstico de diabetes classificou o indivíduo como “DIABÉTICO”, com uma probabilidade estimada de 62.39%. A glicemia elevada e o IMC acima do recomendado são os principais fatores que influenciaram essa classificação, indicando um risco aumentado para o desenvolvimento da doença. A probabilidade de 62.39% sugere que, com base nesses dados, a predição de diabetes é considerada moderada. É fundamental procurar avaliação médica imediata para confirmar o diagnóstico e iniciar o tratamento adequado, lembrando que este resultado não substitui a consulta e o exame clínico de um profissional de saúde.</t>
         </is>
       </c>
     </row>
@@ -510,11 +510,11 @@
         </is>
       </c>
       <c r="G3" t="n">
-        <v>25.11</v>
+        <v>24.66</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Erro ao gerar relatório clínico: Failed to connect to Ollama. Please check that Ollama is downloaded, running and accessible. https://ollama.com/download</t>
+          <t>Com base nos dados fornecidos, o modelo classificou o paciente como NÃO DIABÉTICO com uma probabilidade estimada de 24.66%. A glicose de 90 mg/dL e o IMC de 22 indicam um controle glicêmico e peso saudáveis, sendo fatores que contribuíram para essa classificação. Apesar da baixa probabilidade de 24.66%, é importante ressaltar que essa análise é apenas uma estimativa e não substitui a avaliação completa de um profissional de saúde. Recomendamos fortemente a realização de exames adicionais e acompanhamento médico para garantir a saúde do paciente, pois este resultado não dispensa a consulta e avaliação por um médico.</t>
         </is>
       </c>
     </row>
@@ -540,11 +540,11 @@
         </is>
       </c>
       <c r="G4" t="n">
-        <v>63.07</v>
+        <v>63.03</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Erro ao gerar relatório clínico: Failed to connect to Ollama. Please check that Ollama is downloaded, running and accessible. https://ollama.com/download</t>
+          <t>Com base nos dados fornecidos, o modelo classificou o paciente como diabético com uma probabilidade estimada de 63.03%. A glicemia elevada de 180 mg/dL, juntamente com o IMC de 35, que indica obesidade, foram os principais fatores que influenciaram essa classificação. Essa probabilidade de 63.03% sugere que, com base nesses dados, há uma chance considerável de o paciente ter diabetes. Recomendamos fortemente que o paciente procure avaliação médica completa para confirmar o diagnóstico e iniciar o tratamento adequado. É importante ressaltar que este resultado é apenas uma estimativa e não substitui a avaliação e o julgamento de um profissional de saúde.</t>
         </is>
       </c>
     </row>
@@ -570,11 +570,11 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>51.79</v>
+        <v>51.5</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Erro ao gerar relatório clínico: Failed to connect to Ollama. Please check that Ollama is downloaded, running and accessible. https://ollama.com/download</t>
+          <t>Com base nos dados fornecidos – glicose de 220 mg/dL, IMC de 25 e idade de 32 anos – o modelo classificou o paciente como “DIABÉTICO” com uma probabilidade estimada de 51.50%. A glicemia elevada e o IMC indicam um risco aumentado para o desenvolvimento da doença. A probabilidade de 51.50% sugere que, embora os fatores apontem para a diabetes, ainda existe uma chance de 48.50% de que a condição não seja diagnosticada. Recomendamos fortemente que o paciente procure avaliação médica imediata para confirmar o diagnóstico e iniciar o tratamento adequado. É importante ressaltar que este resultado é apenas uma estimativa e não substitui a avaliação completa de um profissional de saúde.</t>
         </is>
       </c>
     </row>
@@ -600,11 +600,11 @@
         </is>
       </c>
       <c r="G6" t="n">
-        <v>20.62</v>
+        <v>21.18</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Erro ao gerar relatório clínico: Failed to connect to Ollama. Please check that Ollama is downloaded, running and accessible. https://ollama.com/download</t>
+          <t>Com base nos dados fornecidos – glicose de 70 mg/dL, IMC de 25 e idade de 18 anos – o modelo classificou o indivíduo como NÃO DIABÉTICO, com uma probabilidade estimada de 21,18% de não ter a doença. A glicose baixa e a idade jovem são fatores que contribuíram positivamente para essa classificação. No entanto, a probabilidade de 21,18% indica uma pequena chance de diabetes, que ainda merece atenção. Recomendamos um acompanhamento médico para avaliação completa e, se necessário, exames adicionais, lembrando que este resultado não substitui uma consulta médica e diagnóstico profissional.</t>
         </is>
       </c>
     </row>

</xml_diff>